<commit_message>
added duplicate prevention in excel report
</commit_message>
<xml_diff>
--- a/output/reports/request_report.xlsx
+++ b/output/reports/request_report.xlsx
@@ -417,15 +417,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -451,10 +452,15 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Processed at</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
@@ -483,10 +489,15 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>2026-09-14 17:58:10</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Processed</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Document generated: REQ-0001_student_certificate.docx</t>
         </is>
@@ -515,10 +526,15 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>2026-09-14 17:58:10</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Processed</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Document generated: REQ-0002_scholarship_certificate.docx</t>
         </is>
@@ -547,10 +563,15 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>2026-09-14 17:58:10</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Student ID not found: ST9999</t>
         </is>
@@ -579,10 +600,15 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>2026-09-14 17:58:10</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Invalid student status: suspended</t>
         </is>
@@ -611,10 +637,15 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>2026-09-14 17:58:10</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Processed</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Document generated: REQ-0005_student_certificate.docx</t>
         </is>

</xml_diff>